<commit_message>
Datos OB: v4 final (eolica optimista, topes 10, vida_util) y topes 10 en la v3
- Mina_modelo_v4: perfil eolico optimista (norte 7,56 h-eq/dia, centro 5,33),
  topes de solar, eolica y BESS en 10 y columna vida_util (solar 35, eolica 25,
  BESS 20) para el valor residual; tasa 8 %. Se quita la Produccion_escalada
  vieja.
- Mina_modelo (v3): g_max y h_max de 2 a 10 en los casos con generacion, y datos
  de Produccion_escalada20 (1C).
- Mina_modelo_v4_vr y Mina_modelo_v4_machali: pruebas de valor residual y de
  precio variable (Machali) en el caso centro.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Resultados_finales_tesis/Mina_modelo/Produccion_base/zona_centro/05C/P_red_gen_bat/elmo_data.xlsx
+++ b/data/Resultados_finales_tesis/Mina_modelo/Produccion_base/zona_centro/05C/P_red_gen_bat/elmo_data.xlsx
@@ -3312,7 +3312,7 @@
         <v>500</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -3339,7 +3339,7 @@
         <v>500</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -3478,7 +3478,7 @@
         <v>1000</v>
       </c>
       <c r="I3" s="34" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>